<commit_message>
Admin update: Rates updated
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
   <si>
     <t>H001</t>
   </si>
@@ -36,9 +36,6 @@
     <t>Luxury Rose Gold Pull</t>
   </si>
   <si>
-    <t>Limited</t>
-  </si>
-  <si>
     <t>M010</t>
   </si>
   <si>
@@ -49,9 +46,6 @@
   </si>
   <si>
     <t>Pooja Mandir Knob</t>
-  </si>
-  <si>
-    <t>Out of Stock</t>
   </si>
   <si>
     <t>G009</t>
@@ -452,22 +446,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -507,15 +501,15 @@
         <v>3</v>
       </c>
       <c r="F3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
       </c>
       <c r="C4">
         <v>6000</v>
@@ -524,7 +518,7 @@
         <v>5500</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="s">
         <v>2</v>
@@ -532,10 +526,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
       <c r="C5">
         <v>500</v>
@@ -544,18 +538,18 @@
         <v>450</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C6">
         <v>4000</v>
@@ -564,7 +558,7 @@
         <v>3200</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F6" t="s">
         <v>2</v>

</xml_diff>